<commit_message>
doc(JDT): maj du JDT
</commit_message>
<xml_diff>
--- a/Doc Backend/Journal-de-Travail_LäuppiRyan-Backend.xlsx
+++ b/Doc Backend/Journal-de-Travail_LäuppiRyan-Backend.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pa33xxl\Documents\GitHub\Passion-Lecture\Doc Backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C497E7DD-486A-44FD-916A-FF0A0EDD3EE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2480DE7B-898D-4283-8CA9-7C556855E677}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="39">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -152,6 +152,12 @@
   </si>
   <si>
     <t>M.Charmier m'a aidé à chercher le JDT mais il à vraiment disparu</t>
+  </si>
+  <si>
+    <t>J'ai changé seeders pour qu'il n'y ait plus d'erreurs et que les données soient en database</t>
+  </si>
+  <si>
+    <t>J'ai commencé le comment controller</t>
   </si>
 </sst>
 </file>
@@ -1159,10 +1165,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>70</c:v>
+                  <c:v>75</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>90</c:v>
+                  <c:v>160</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2014,10 +2020,10 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.4375</c:v>
+                  <c:v>0.31914893617021278</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.5625</c:v>
+                  <c:v>0.68085106382978722</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -4258,7 +4264,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>2 heures 40 minutes</v>
+        <v>3 heures 55 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4275,11 +4281,11 @@
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>100</v>
+        <v>175</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>160</v>
+        <v>235</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4457,7 +4463,7 @@
       </c>
       <c r="C12" s="31"/>
       <c r="D12" s="32">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E12" s="33" t="s">
         <v>13</v>
@@ -4477,15 +4483,23 @@
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="63" t="str">
+      <c r="A13" s="63">
         <f>IF(ISBLANK(B13),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B13))</f>
-        <v/>
-      </c>
-      <c r="B13" s="34"/>
+        <v>19</v>
+      </c>
+      <c r="B13" s="34">
+        <v>46147</v>
+      </c>
       <c r="C13" s="35"/>
-      <c r="D13" s="36"/>
-      <c r="E13" s="37"/>
-      <c r="F13" s="23"/>
+      <c r="D13" s="36">
+        <v>40</v>
+      </c>
+      <c r="E13" s="37" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" s="23" t="s">
+        <v>37</v>
+      </c>
       <c r="G13" s="40"/>
       <c r="N13">
         <v>6</v>
@@ -4495,15 +4509,23 @@
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="62" t="str">
+      <c r="A14" s="62">
         <f>IF(ISBLANK(B14),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B14))</f>
-        <v/>
-      </c>
-      <c r="B14" s="30"/>
+        <v>19</v>
+      </c>
+      <c r="B14" s="30">
+        <v>46147</v>
+      </c>
       <c r="C14" s="31"/>
-      <c r="D14" s="32"/>
-      <c r="E14" s="33"/>
-      <c r="F14" s="23"/>
+      <c r="D14" s="32">
+        <v>30</v>
+      </c>
+      <c r="E14" s="33" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" s="23" t="s">
+        <v>38</v>
+      </c>
       <c r="G14" s="39"/>
       <c r="N14">
         <v>7</v>
@@ -10884,11 +10906,11 @@
       </c>
       <c r="B6">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E6,'Journal de travail'!$D$7:$D$532)</f>
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="C6">
         <f t="shared" ref="C6:C10" si="0">SUM(A6:B6)</f>
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="E6" s="70" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10896,11 +10918,11 @@
       </c>
       <c r="F6" s="71" t="str">
         <f>QUOTIENT(SUM(A6:B6),60)&amp;" h "&amp;TEXT(MOD(SUM(A6:B6),60), "00")&amp;" min"</f>
-        <v>1 h 10 min</v>
+        <v>1 h 15 min</v>
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>0.4375</v>
+        <v>0.31914893617021278</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10921,11 +10943,11 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>90</v>
+        <v>160</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10933,11 +10955,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>1 h 30 min</v>
+        <v>2 h 40 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.5625</v>
+        <v>0.68085106382978722</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11067,22 +11089,22 @@
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>100</v>
+        <v>175</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>160</v>
+        <v>235</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>28</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>2 h 40 min</v>
+        <v>3 h 55 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>2.9629629629629631E-2</v>
+        <v>4.3518518518518519E-2</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>28</v>
@@ -11121,6 +11143,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005B1120F001D1794FAA6F4057E3355991" ma:contentTypeVersion="10" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="5bf905bc6027d3a3176cf398b6d748a7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f20a0681-8b2f-4a46-9dab-cf1520193f81" xmlns:ns3="932fafb7-d8e0-4a14-bee3-33aad5c71309" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="cdc8923a5f0a5cb2ad217e59a32ed26c" ns2:_="" ns3:_="">
     <xsd:import namespace="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
@@ -11309,17 +11342,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -11330,6 +11352,17 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
+    <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EB23EBB1-226D-48F9-BD4F-72DBF2899D35}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11348,17 +11381,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
-    <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>

</xml_diff>